<commit_message>
Flag row 5 (Failed to fit screws) Remark: plant Effect list may be incomplete
Added a generic manual_review_note mechanism to build_remark() - a
human-added flag rendered as its own Remark bullet, separate from the
LLM's own output, for cases the AI can't judge on its own (here: a
gap in the plant's source data, not a GPT-5 scoring error - see chat
discussion). Applied only to the 'Failed to fit screws / not
maintained gap' row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MG2nzeeWa5SnWqcTDjXsda
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode_gpt5.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode_gpt5.xlsx
@@ -3063,7 +3063,7 @@
       <c r="AS25" s="223" t="n"/>
       <c r="AT25" s="223" t="n"/>
     </row>
-    <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
+    <row r="26" ht="157.5" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
       <c r="C26" s="211" t="n"/>
       <c r="D26" s="210" t="n"/>
@@ -3160,12 +3160,13 @@
       </c>
       <c r="AT26" s="223" t="inlineStr">
         <is>
-          <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
+          <t>- REVIEWER NOTE: Plant listed only cosmetic/NVH End User effects for this row (lens crack, LED burnout, water ingress, rattling, discomfort) - no beam-alignment/visibility/accident-risk option, unlike the near-identical 'Prefit bolts' step (same mounting joint) which lists those and scored S=10. If loose/missing screws can also misalign the beam, add that effect to this row's own Effect cell in the plant's source Excel so AI severity reflects it; do not change AI/prompt logic to compensate - broadening the effect list plant-wide risks re-inflating severity on unrelated rows (a documented past failure mode of this pipeline).
+- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
 - Cause/Mode mismatch: The recorded Cause addresses only gap uniformity between headlamp edge and fender and does not explain the merged Mode’s "failed to fit screws" sub-mode.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="156" customFormat="1" customHeight="1" s="13">
+    <row r="27" ht="157.5" customFormat="1" customHeight="1" s="13">
       <c r="B27" s="210" t="n"/>
       <c r="C27" s="211" t="n"/>
       <c r="D27" s="210" t="n"/>

</xml_diff>

<commit_message>
Build final merge-mode Excel with AI Review findings merged in
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode_gpt5.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode_gpt5.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="AU26" s="223" t="inlineStr">
         <is>
-          <t>Plant listed only cosmetic/NVH End User effects for this row (lens crack, LED burnout, water ingress, rattling, discomfort) - no beam-alignment/visibility/accident-risk option, unlike the near-identical 'Prefit bolts' step (same mounting joint) which lists those and scored S=10. If loose/missing screws can also misalign the beam, add that effect to this row's own Effect cell in the plant's source Excel so AI severity reflects it; do not change AI/prompt logic to compensate - broadening the effect list plant-wide risks re-inflating severity on unrelated rows (a documented past failure mode of this pipeline).</t>
+          <t>Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
         </is>
       </c>
       <c r="AV26" s="223" t="inlineStr"/>
@@ -3969,7 +3969,11 @@
           <t>- Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
-      <c r="AU28" s="223" t="inlineStr"/>
+      <c r="AU28" s="223" t="inlineStr">
+        <is>
+          <t>Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
       <c r="AV28" s="223" t="inlineStr"/>
     </row>
     <row r="29" ht="225" customFormat="1" customHeight="1" s="13">
@@ -4053,7 +4057,11 @@
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
-      <c r="AU29" s="223" t="inlineStr"/>
+      <c r="AU29" s="223" t="inlineStr">
+        <is>
+          <t>Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
       <c r="AV29" s="223" t="inlineStr"/>
     </row>
     <row r="30" customFormat="1" s="18"/>

</xml_diff>